<commit_message>
Store the Results status formula as a dynamic-array formula
The owner's Excel showed the new Results A3 formula as
=@ResultsStatusText(...). Excel 365 opens a formula stored the legacy way
that calls a VBA function with whole-column ranges as an implicit-
intersection formula and shows the @ operator. The function returns one
text, so the value was right, but the @ looks like an error and the owner
removed it by hand.

The template now stores A3 as Excel 365 saves a dynamic-array formula:
the cell carries cm="1" and an array formula over A3, and a new
xl/metadata.xml part (XLDAPR dynamic-array properties) is related from
the workbook and declared in [Content_Types].xml. Nothing else in the
package changes. Template SHA-256 c75d8568...ea441b4ca.

Validated: python tools/check.py (all gates pass, including the
committed-workbook check); openpyxl reads A3 as an array formula and
LibreOffice converts the file. Excel not run on this commit.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -49,6 +49,28 @@
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -23461,8 +23483,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="str">
-        <f>ResultsStatusText(SACCR_RunInputs,NettingSets!$A:$N,Trades!$A:$W,Params!$A:$H)</f>
+      <c r="A3" s="30" t="str" cm="1">
+        <f t="array" ref="A3">ResultsStatusText(SACCR_RunInputs,NettingSets!$A:$N,Trades!$A:$W,Params!$A:$H)</f>
         <v>No results: press Run SA-CCR.</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Center every template cell vertically
Owner's request after verifying the status cell: all cells vertically
centered. Every cell format in xl/styles.xml (the 55 cellXfs and the base
cellStyleXfs entry) now has vertical="center", replacing "top" where it
was set; horizontal alignment, wrapping and every other property are
unchanged, and no cell, formula or name changes. Template SHA-256
14db8088...564184af.

Validated: python tools/check.py (all gates pass, including the
committed-workbook check); every cell in the sheet XML references a
centered format; the file opens in openpyxl and converts headless in
LibreOffice. Excel not run on this commit.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -3009,101 +3009,175 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="55">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="173" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="174" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="175" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="175" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">

</xml_diff>

<commit_message>
Show out-of-date results with a formula so Undo keeps working (#89)
Follow-up to #85 (#36). The out-of-date marker was written to Results A2
by a macro on sheet activation, which cleared Excel's undo history.
Results A3 now holds =ResultsStatusText(SACCR_RunInputs, NettingSets!$A:$N,
Trades!$A:$W, Params!$A:$H), stored as a dynamic-array formula and
recalculated by Excel on an input edit or a run, red when OUT OF DATE.
The hidden name SACCR_RunInputs always exists and is emptied rather than
deleted; FlagStaleResults and the shResults activation code are removed.
Every template cell is vertically centred. Includes release/1.0.0's #92
template text.

Validated: python tools/check.py. Verified in Excel by the owner on a
fresh workbook: TEST_MainState 10 cases / 75 checks PASS, TEST_Harness
PASS, Run SA-CCR unchanged (62 of 65, EAD 425.197.518); by hand, an MtM
edit turns A3 OUT OF DATE and Ctrl+Z restores both the value and A3; no
@ in A3; all cells vertically centred.
</commit_message>
<xml_diff>
--- a/src/workbook/SACCR_Template.xlsx
+++ b/src/workbook/SACCR_Template.xlsx
@@ -42,12 +42,35 @@
     <definedName name="MultiplierFloor">Params!$C$8</definedName>
     <definedName name="Regime">Params!$C$22</definedName>
     <definedName name="ReportingCcy">Params!$C$6</definedName>
+    <definedName name="SACCR_RunInputs" hidden="1">""</definedName>
     <definedName name="SDFloorBD">Params!$C$12</definedName>
     <definedName name="SF_Table">Params!$A$27:$I$53</definedName>
     <definedName name="VolatilityFactor">Params!$C$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2986,101 +3009,175 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="55">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="172" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="173" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="173" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="171" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="174" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="173" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="174" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="175" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="175" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment vertical="center" horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -23459,6 +23556,12 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="30" t="str" cm="1">
+        <f t="array" ref="A3">ResultsStatusText(SACCR_RunInputs,NettingSets!$A:$N,Trades!$A:$W,Params!$A:$H)</f>
+        <v>No results: press Run SA-CCR.</v>
+      </c>
+    </row>
     <row r="4" spans="1:28" ht="42" customHeight="1">
       <c r="A4" s="31" t="s">
         <v>259</v>
@@ -23942,6 +24045,11 @@
       <c r="AA20" s="36"/>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="A3">
+    <cfRule type="beginsWith" dxfId="1" priority="1" operator="beginsWith" text="OUT OF DATE">
+      <formula>LEFT(A3,LEN("OUT OF DATE"))="OUT OF DATE"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
   <legacyDrawing r:id="rId1"/>

</xml_diff>